<commit_message>
Correlaciones con rotación - FAMD
</commit_message>
<xml_diff>
--- a/271025_Results_Med/famd/correlations_famd_29102025.xlsx
+++ b/271025_Results_Med/famd/correlations_famd_29102025.xlsx
@@ -1,21 +1,221 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20374"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Portatil\Desktop\Natura\271025_Results_Med\famd\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD14A50-EE76-42CF-8316-D0BCBEEDDF34}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="20" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+  <si>
+    <t>variable</t>
+  </si>
+  <si>
+    <t>dim1.rot</t>
+  </si>
+  <si>
+    <t>dim2.rot</t>
+  </si>
+  <si>
+    <t>dim3.rot</t>
+  </si>
+  <si>
+    <t>dim4.rot</t>
+  </si>
+  <si>
+    <t>dim5.rot</t>
+  </si>
+  <si>
+    <t>dim6.rot</t>
+  </si>
+  <si>
+    <t>dim7.rot</t>
+  </si>
+  <si>
+    <t>dim8.rot</t>
+  </si>
+  <si>
+    <t>dim9.rot</t>
+  </si>
+  <si>
+    <t>dim10.rot</t>
+  </si>
+  <si>
+    <t>dim11.rot</t>
+  </si>
+  <si>
+    <t>dim12.rot</t>
+  </si>
+  <si>
+    <t>p1edad</t>
+  </si>
+  <si>
+    <t>p24</t>
+  </si>
+  <si>
+    <t>p28_importancia_costo_compra</t>
+  </si>
+  <si>
+    <t>p28_importancia_costo_uso</t>
+  </si>
+  <si>
+    <t>p28_importancia_comodidad</t>
+  </si>
+  <si>
+    <t>p28_importancia_tiempo</t>
+  </si>
+  <si>
+    <t>p28_importancia_riesgo_robo</t>
+  </si>
+  <si>
+    <t>p28_importancia_riesgo_acoso</t>
+  </si>
+  <si>
+    <t>p28_importancia_discriminacion</t>
+  </si>
+  <si>
+    <t>p28_importancia_emisiones</t>
+  </si>
+  <si>
+    <t>p28_importancia_siniestralidad</t>
+  </si>
+  <si>
+    <t>p32_contaminacion_likert</t>
+  </si>
+  <si>
+    <t>p36_influencia_amigos</t>
+  </si>
+  <si>
+    <t>p37_influencia_familia</t>
+  </si>
+  <si>
+    <t>tiempo_total</t>
+  </si>
+  <si>
+    <t>edad_r2</t>
+  </si>
+  <si>
+    <t>pais</t>
+  </si>
+  <si>
+    <t>p3_agregado</t>
+  </si>
+  <si>
+    <t>p5_agregado</t>
+  </si>
+  <si>
+    <t>p7_agregado</t>
+  </si>
+  <si>
+    <t>p8_agregado</t>
+  </si>
+  <si>
+    <t>p9_estrato3</t>
+  </si>
+  <si>
+    <t>p40</t>
+  </si>
+  <si>
+    <t>p13</t>
+  </si>
+  <si>
+    <t>p14</t>
+  </si>
+  <si>
+    <t>p15_autos_agregado</t>
+  </si>
+  <si>
+    <t>p15_1_autos_propios_agregado</t>
+  </si>
+  <si>
+    <t>p16_motos_agregado</t>
+  </si>
+  <si>
+    <t>p16_1_motos_propias_agregado</t>
+  </si>
+  <si>
+    <t>p17_modo_agregado</t>
+  </si>
+  <si>
+    <t>cilindraje_auto_agregado</t>
+  </si>
+  <si>
+    <t>cilindraje_moto_agregado</t>
+  </si>
+  <si>
+    <t>modelo_vehiculo_agregado</t>
+  </si>
+  <si>
+    <t>p19comuna</t>
+  </si>
+  <si>
+    <t>p22</t>
+  </si>
+  <si>
+    <t>p23_agregado</t>
+  </si>
+  <si>
+    <t>p26_agregado</t>
+  </si>
+  <si>
+    <t>p29_modo_ideal_agregado</t>
+  </si>
+  <si>
+    <t>p30_razon_no_uso_agregado</t>
+  </si>
+  <si>
+    <t>p31_fuente_contaminacion_agregada</t>
+  </si>
+  <si>
+    <t>p33_modo_contaminante_agregado</t>
+  </si>
+  <si>
+    <t>p35_razon_agregada</t>
+  </si>
+  <si>
+    <t>p38p38_1</t>
+  </si>
+  <si>
+    <t>p38p38_2</t>
+  </si>
+  <si>
+    <t>p38p38_3</t>
+  </si>
+  <si>
+    <t>p38p38_4</t>
+  </si>
+  <si>
+    <t>p38p38_5</t>
+  </si>
+  <si>
+    <t>p38p38_6</t>
+  </si>
+  <si>
+    <t>p38p38_7</t>
+  </si>
+  <si>
+    <t>p38p38_99</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -32,12 +232,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -52,22 +258,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -109,7 +325,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -141,9 +357,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -175,6 +409,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -350,149 +602,122 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M51"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="35.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>dim1.rot</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>dim2.rot</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>dim3.rot</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>dim4.rot</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>dim5.rot</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>dim6.rot</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>dim7.rot</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>dim8.rot</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>dim9.rot</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>dim10.rot</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>dim11.rot</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>dim12.rot</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>p1edad</t>
-        </is>
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
-        <v>0.0384</v>
+        <v>3.8399999999999997E-2</v>
       </c>
       <c r="C2">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="D2">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="E2">
-        <v>0.7028</v>
+        <v>0.70279999999999998</v>
       </c>
       <c r="F2">
-        <v>0.0039</v>
+        <v>3.8999999999999998E-3</v>
       </c>
       <c r="G2">
-        <v>0.0057</v>
+        <v>5.7000000000000002E-3</v>
       </c>
       <c r="H2">
-        <v>0.0103</v>
+        <v>1.03E-2</v>
       </c>
       <c r="I2">
-        <v>0.0008</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="J2">
-        <v>0.0051</v>
+        <v>5.1000000000000004E-3</v>
       </c>
       <c r="K2">
-        <v>0.005</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="L2">
-        <v>0.0061</v>
+        <v>6.1000000000000004E-3</v>
       </c>
       <c r="M2">
-        <v>0.0028</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>p24</t>
-        </is>
+        <v>2.8E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
       </c>
       <c r="B3">
-        <v>0.0633</v>
+        <v>6.3299999999999995E-2</v>
       </c>
       <c r="C3">
-        <v>0.0474</v>
+        <v>4.7399999999999998E-2</v>
       </c>
       <c r="D3">
-        <v>0.0044</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="E3">
-        <v>0.0005999999999999999</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="F3">
-        <v>0.0019</v>
+        <v>1.9E-3</v>
       </c>
       <c r="G3">
-        <v>0.0115</v>
+        <v>1.15E-2</v>
       </c>
       <c r="H3">
-        <v>0.0014</v>
+        <v>1.4E-3</v>
       </c>
       <c r="I3">
-        <v>0.0111</v>
+        <v>1.11E-2</v>
       </c>
       <c r="J3">
         <v>0.1028</v>
@@ -501,508 +726,484 @@
         <v>0</v>
       </c>
       <c r="L3">
-        <v>0.033</v>
+        <v>3.3000000000000002E-2</v>
       </c>
       <c r="M3">
-        <v>0.0252</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>p28_importancia_costo_compra</t>
-        </is>
+        <v>2.52E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>15</v>
       </c>
       <c r="B4">
-        <v>0.0034</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="C4">
-        <v>0.0372</v>
+        <v>3.7199999999999997E-2</v>
       </c>
       <c r="D4">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="E4">
-        <v>0.0031</v>
+        <v>3.0999999999999999E-3</v>
       </c>
       <c r="F4">
-        <v>0.1712</v>
+        <v>0.17119999999999999</v>
       </c>
       <c r="G4">
-        <v>0.0218</v>
+        <v>2.18E-2</v>
       </c>
       <c r="H4">
-        <v>0.0005</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="I4">
-        <v>0.0222</v>
+        <v>2.2200000000000001E-2</v>
       </c>
       <c r="J4">
-        <v>0.0564</v>
+        <v>5.6399999999999999E-2</v>
       </c>
       <c r="K4">
-        <v>0.009599999999999999</v>
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="L4">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="M4">
-        <v>0.0083</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>p28_importancia_costo_uso</t>
-        </is>
+        <v>8.3000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>16</v>
       </c>
       <c r="B5">
-        <v>0.0488</v>
+        <v>4.8800000000000003E-2</v>
       </c>
       <c r="C5">
-        <v>0.0167</v>
+        <v>1.67E-2</v>
       </c>
       <c r="D5">
-        <v>0.0287</v>
+        <v>2.87E-2</v>
       </c>
       <c r="E5">
-        <v>0.0024</v>
+        <v>2.3999999999999998E-3</v>
       </c>
       <c r="F5">
-        <v>0.1569</v>
+        <v>0.15690000000000001</v>
       </c>
       <c r="G5">
-        <v>0.0071</v>
+        <v>7.1000000000000004E-3</v>
       </c>
       <c r="H5">
-        <v>0.0014</v>
+        <v>1.4E-3</v>
       </c>
       <c r="I5">
-        <v>0.0043</v>
+        <v>4.3E-3</v>
       </c>
       <c r="J5">
-        <v>0.0401</v>
+        <v>4.0099999999999997E-2</v>
       </c>
       <c r="K5">
-        <v>0.0218</v>
+        <v>2.18E-2</v>
       </c>
       <c r="L5">
-        <v>0.0025</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="M5">
-        <v>0.0028</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>p28_importancia_comodidad</t>
-        </is>
+        <v>2.8E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>17</v>
       </c>
       <c r="B6">
-        <v>0.0221</v>
+        <v>2.2100000000000002E-2</v>
       </c>
       <c r="C6">
-        <v>0.0265</v>
+        <v>2.6499999999999999E-2</v>
       </c>
       <c r="D6">
-        <v>0.0063</v>
+        <v>6.3E-3</v>
       </c>
       <c r="E6">
-        <v>0.0047</v>
+        <v>4.7000000000000002E-3</v>
       </c>
       <c r="F6">
-        <v>0.0594</v>
+        <v>5.9400000000000001E-2</v>
       </c>
       <c r="G6">
-        <v>0.0005999999999999999</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>0.0013</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="J6">
-        <v>0.2153</v>
+        <v>0.21529999999999999</v>
       </c>
       <c r="K6">
-        <v>0.0098</v>
+        <v>9.7999999999999997E-3</v>
       </c>
       <c r="L6">
-        <v>0.0304</v>
+        <v>3.04E-2</v>
       </c>
       <c r="M6">
-        <v>0.008699999999999999</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>p28_importancia_tiempo</t>
-        </is>
+        <v>8.6999999999999994E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>18</v>
       </c>
       <c r="B7">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="C7">
-        <v>0.0418</v>
+        <v>4.1799999999999997E-2</v>
       </c>
       <c r="D7">
-        <v>0.0017</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="E7">
-        <v>0.0013</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="F7">
-        <v>0.0689</v>
+        <v>6.8900000000000003E-2</v>
       </c>
       <c r="G7">
-        <v>0.0045</v>
+        <v>4.4999999999999997E-3</v>
       </c>
       <c r="H7">
-        <v>0.0013</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="I7">
-        <v>0.0058</v>
+        <v>5.7999999999999996E-3</v>
       </c>
       <c r="J7">
-        <v>0.1957</v>
+        <v>0.19570000000000001</v>
       </c>
       <c r="K7">
-        <v>0.0196</v>
+        <v>1.9599999999999999E-2</v>
       </c>
       <c r="L7">
-        <v>0.0383</v>
+        <v>3.8300000000000001E-2</v>
       </c>
       <c r="M7">
-        <v>0.0045</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>p28_importancia_riesgo_robo</t>
-        </is>
+        <v>4.4999999999999997E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>19</v>
       </c>
       <c r="B8">
-        <v>0.0043</v>
+        <v>4.3E-3</v>
       </c>
       <c r="C8">
-        <v>0.0044</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="D8">
-        <v>0.0008</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="E8">
-        <v>0.0015</v>
+        <v>1.5E-3</v>
       </c>
       <c r="F8">
         <v>0.5665</v>
       </c>
       <c r="G8">
-        <v>0.0009</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
-        <v>0.0012</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="J8">
-        <v>0.0002</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="K8">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="L8">
-        <v>0.0005999999999999999</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="M8">
-        <v>0.0001</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>p28_importancia_riesgo_acoso</t>
-        </is>
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>20</v>
       </c>
       <c r="B9">
-        <v>0.0108</v>
+        <v>1.0800000000000001E-2</v>
       </c>
       <c r="C9">
-        <v>0.0092</v>
+        <v>9.1999999999999998E-3</v>
       </c>
       <c r="D9">
-        <v>0.0022</v>
+        <v>2.2000000000000001E-3</v>
       </c>
       <c r="E9">
-        <v>0.0032</v>
+        <v>3.2000000000000002E-3</v>
       </c>
       <c r="F9">
-        <v>0.6343</v>
+        <v>0.63429999999999997</v>
       </c>
       <c r="G9">
-        <v>0.0044</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="H9">
-        <v>0.0037</v>
+        <v>3.7000000000000002E-3</v>
       </c>
       <c r="I9">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="J9">
-        <v>0.0008</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="K9">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="L9">
-        <v>0.0009</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="M9">
-        <v>0.0003</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>p28_importancia_discriminacion</t>
-        </is>
+        <v>2.9999999999999997E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
       <c r="B10">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="C10">
-        <v>0.0005999999999999999</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="D10">
-        <v>0.0012</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="E10">
-        <v>0.0023</v>
+        <v>2.3E-3</v>
       </c>
       <c r="F10">
-        <v>0.5152</v>
+        <v>0.51519999999999999</v>
       </c>
       <c r="G10">
-        <v>0.0047</v>
+        <v>4.7000000000000002E-3</v>
       </c>
       <c r="H10">
-        <v>0.0033</v>
+        <v>3.3E-3</v>
       </c>
       <c r="I10">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="J10">
-        <v>0.0007</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="K10">
-        <v>0.0005</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="L10">
-        <v>0.007</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="M10">
         <v>0</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>p28_importancia_emisiones</t>
-        </is>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11">
         <v>0</v>
       </c>
       <c r="C11">
-        <v>0.0009</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="D11">
-        <v>0.0009</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="E11">
-        <v>0.0016</v>
+        <v>1.6000000000000001E-3</v>
       </c>
       <c r="F11">
-        <v>0.5861</v>
+        <v>0.58609999999999995</v>
       </c>
       <c r="G11">
-        <v>0.0044</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="H11">
-        <v>0.0008</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="I11">
-        <v>0.0012</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="J11">
-        <v>0.0029</v>
+        <v>2.8999999999999998E-3</v>
       </c>
       <c r="K11">
-        <v>0.0048</v>
+        <v>4.7999999999999996E-3</v>
       </c>
       <c r="L11">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="M11">
-        <v>0.0001</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>p28_importancia_siniestralidad</t>
-        </is>
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>23</v>
       </c>
       <c r="B12">
-        <v>0.0217</v>
+        <v>2.1700000000000001E-2</v>
       </c>
       <c r="C12">
-        <v>0.0336</v>
+        <v>3.3599999999999998E-2</v>
       </c>
       <c r="D12">
-        <v>0.0018</v>
+        <v>1.8E-3</v>
       </c>
       <c r="E12">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="F12">
         <v>0.4773</v>
       </c>
       <c r="G12">
-        <v>0.0133</v>
+        <v>1.3299999999999999E-2</v>
       </c>
       <c r="H12">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="I12">
-        <v>0.0007</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="J12">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="K12">
-        <v>0.0098</v>
+        <v>9.7999999999999997E-3</v>
       </c>
       <c r="L12">
-        <v>0.0077</v>
+        <v>7.7000000000000002E-3</v>
       </c>
       <c r="M12">
         <v>0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>p32_contaminacion_likert</t>
-        </is>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>24</v>
       </c>
       <c r="B13">
-        <v>0.0026</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="C13">
-        <v>0.0115</v>
+        <v>1.15E-2</v>
       </c>
       <c r="D13">
-        <v>0.0022</v>
+        <v>2.2000000000000001E-3</v>
       </c>
       <c r="E13">
-        <v>0.0411</v>
+        <v>4.1099999999999998E-2</v>
       </c>
       <c r="F13">
-        <v>0.0017</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
       <c r="H13">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="I13">
-        <v>0.0072</v>
+        <v>7.1999999999999998E-3</v>
       </c>
       <c r="J13">
-        <v>0.0286</v>
+        <v>2.86E-2</v>
       </c>
       <c r="K13">
-        <v>0.0179</v>
+        <v>1.7899999999999999E-2</v>
       </c>
       <c r="L13">
         <v>0.1653</v>
       </c>
       <c r="M13">
-        <v>0.0294</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>p36_influencia_amigos</t>
-        </is>
+        <v>2.9399999999999999E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14">
-        <v>0.0284</v>
+        <v>2.8400000000000002E-2</v>
       </c>
       <c r="C14">
-        <v>0.0015</v>
+        <v>1.5E-3</v>
       </c>
       <c r="D14">
-        <v>0.0179</v>
+        <v>1.7899999999999999E-2</v>
       </c>
       <c r="E14">
-        <v>0.0333</v>
+        <v>3.3300000000000003E-2</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
       <c r="G14">
-        <v>0.0318</v>
+        <v>3.1800000000000002E-2</v>
       </c>
       <c r="H14">
-        <v>0.0002</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="I14">
-        <v>0.0002</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="J14">
-        <v>0.3229</v>
+        <v>0.32290000000000002</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>0.0183</v>
+        <v>1.83E-2</v>
       </c>
       <c r="M14">
-        <v>0.0011</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>p37_influencia_familia</t>
-        </is>
+        <v>1.1000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>26</v>
       </c>
       <c r="B15">
-        <v>0.0304</v>
+        <v>3.04E-2</v>
       </c>
       <c r="C15">
-        <v>0.0118</v>
+        <v>1.18E-2</v>
       </c>
       <c r="D15">
-        <v>0.0073</v>
+        <v>7.3000000000000001E-3</v>
       </c>
       <c r="E15">
-        <v>0.0164</v>
+        <v>1.6400000000000001E-2</v>
       </c>
       <c r="F15">
-        <v>0.0005999999999999999</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="G15">
-        <v>0.019</v>
+        <v>1.9E-2</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -1011,999 +1212,953 @@
         <v>0</v>
       </c>
       <c r="J15">
-        <v>0.3476</v>
+        <v>0.34760000000000002</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>0.005</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="M15">
-        <v>0.004</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>tiempo_total</t>
-        </is>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>27</v>
       </c>
       <c r="B16">
-        <v>0.1765</v>
+        <v>0.17649999999999999</v>
       </c>
       <c r="C16">
-        <v>0.0049</v>
+        <v>4.8999999999999998E-3</v>
       </c>
       <c r="D16">
-        <v>0.0413</v>
+        <v>4.1300000000000003E-2</v>
       </c>
       <c r="E16">
-        <v>0.0012</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="F16">
-        <v>0.0038</v>
+        <v>3.8E-3</v>
       </c>
       <c r="G16">
         <v>0.01</v>
       </c>
       <c r="H16">
-        <v>0.0025</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="I16">
-        <v>0.1785</v>
+        <v>0.17849999999999999</v>
       </c>
       <c r="J16">
-        <v>0.0049</v>
+        <v>4.8999999999999998E-3</v>
       </c>
       <c r="K16">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="L16">
-        <v>0.0379</v>
+        <v>3.7900000000000003E-2</v>
       </c>
       <c r="M16">
         <v>0</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>edad_r2</t>
-        </is>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>28</v>
       </c>
       <c r="B17">
-        <v>0.0707</v>
+        <v>7.0699999999999999E-2</v>
       </c>
       <c r="C17">
-        <v>0.0038</v>
+        <v>3.8E-3</v>
       </c>
       <c r="D17">
-        <v>0.0037</v>
+        <v>3.7000000000000002E-3</v>
       </c>
       <c r="E17">
-        <v>0.6457000000000001</v>
+        <v>0.64570000000000005</v>
       </c>
       <c r="F17">
-        <v>0.0072</v>
+        <v>7.1999999999999998E-3</v>
       </c>
       <c r="G17">
         <v>0.1487</v>
       </c>
       <c r="H17">
-        <v>0.0123</v>
+        <v>1.23E-2</v>
       </c>
       <c r="I17">
-        <v>0.0742</v>
+        <v>7.4200000000000002E-2</v>
       </c>
       <c r="J17">
-        <v>0.0049</v>
+        <v>4.8999999999999998E-3</v>
       </c>
       <c r="K17">
-        <v>0.0198</v>
+        <v>1.9800000000000002E-2</v>
       </c>
       <c r="L17">
-        <v>0.0074</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="M17">
-        <v>0.0358</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>pais</t>
-        </is>
+        <v>3.5799999999999998E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>29</v>
       </c>
       <c r="B18">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="C18">
-        <v>0.0014</v>
+        <v>1.4E-3</v>
       </c>
       <c r="D18">
-        <v>0.0123</v>
+        <v>1.23E-2</v>
       </c>
       <c r="E18">
-        <v>0.0193</v>
+        <v>1.9300000000000001E-2</v>
       </c>
       <c r="F18">
-        <v>0.0058</v>
+        <v>5.7999999999999996E-3</v>
       </c>
       <c r="G18">
-        <v>0.0034</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="H18">
-        <v>0.0067</v>
+        <v>6.7000000000000002E-3</v>
       </c>
       <c r="I18">
-        <v>0.0277</v>
+        <v>2.7699999999999999E-2</v>
       </c>
       <c r="J18">
-        <v>0.0138</v>
+        <v>1.38E-2</v>
       </c>
       <c r="K18">
-        <v>0.0274</v>
+        <v>2.7400000000000001E-2</v>
       </c>
       <c r="L18">
-        <v>0.0018</v>
+        <v>1.8E-3</v>
       </c>
       <c r="M18">
-        <v>0.0259</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>p3_agregado</t>
-        </is>
+        <v>2.5899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>30</v>
       </c>
       <c r="B19">
-        <v>0.0032</v>
+        <v>3.2000000000000002E-3</v>
       </c>
       <c r="C19">
-        <v>0.0529</v>
+        <v>5.2900000000000003E-2</v>
       </c>
       <c r="D19">
-        <v>0.0102</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="E19">
-        <v>0.0468</v>
+        <v>4.6800000000000001E-2</v>
       </c>
       <c r="F19">
-        <v>0.0395</v>
+        <v>3.95E-2</v>
       </c>
       <c r="G19">
-        <v>0.0602</v>
+        <v>6.0199999999999997E-2</v>
       </c>
       <c r="H19">
-        <v>0.0203</v>
+        <v>2.0299999999999999E-2</v>
       </c>
       <c r="I19">
-        <v>0.0054</v>
+        <v>5.4000000000000003E-3</v>
       </c>
       <c r="J19">
-        <v>0.0703</v>
+        <v>7.0300000000000001E-2</v>
       </c>
       <c r="K19">
-        <v>0.009900000000000001</v>
+        <v>9.9000000000000008E-3</v>
       </c>
       <c r="L19">
-        <v>0.0034</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="M19">
         <v>0.1158</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>p5_agregado</t>
-        </is>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>31</v>
       </c>
       <c r="B20">
-        <v>0.0297</v>
+        <v>2.9700000000000001E-2</v>
       </c>
       <c r="C20">
-        <v>0.0113</v>
+        <v>1.1299999999999999E-2</v>
       </c>
       <c r="D20">
-        <v>0.1456</v>
+        <v>0.14560000000000001</v>
       </c>
       <c r="E20">
         <v>0.1925</v>
       </c>
       <c r="F20">
-        <v>0.0017</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="G20">
-        <v>0.202</v>
+        <v>0.20200000000000001</v>
       </c>
       <c r="H20">
-        <v>0.013</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="I20">
-        <v>0.0613</v>
+        <v>6.13E-2</v>
       </c>
       <c r="J20">
-        <v>0.0475</v>
+        <v>4.7500000000000001E-2</v>
       </c>
       <c r="K20">
-        <v>0.0238</v>
+        <v>2.3800000000000002E-2</v>
       </c>
       <c r="L20">
-        <v>0.0732</v>
+        <v>7.3200000000000001E-2</v>
       </c>
       <c r="M20">
-        <v>0.0295</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>p7_agregado</t>
-        </is>
+        <v>2.9499999999999998E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>32</v>
       </c>
       <c r="B21">
         <v>0.123</v>
       </c>
       <c r="C21">
-        <v>0.034</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="D21">
-        <v>0.08989999999999999</v>
+        <v>8.9899999999999994E-2</v>
       </c>
       <c r="E21">
-        <v>0.5803</v>
+        <v>0.58030000000000004</v>
       </c>
       <c r="F21">
-        <v>0.0288</v>
+        <v>2.8799999999999999E-2</v>
       </c>
       <c r="G21">
-        <v>0.1102</v>
+        <v>0.11020000000000001</v>
       </c>
       <c r="H21">
-        <v>0.0192</v>
+        <v>1.9199999999999998E-2</v>
       </c>
       <c r="I21">
-        <v>0.2809</v>
+        <v>0.28089999999999998</v>
       </c>
       <c r="J21">
-        <v>0.0528</v>
+        <v>5.28E-2</v>
       </c>
       <c r="K21">
-        <v>0.0726</v>
+        <v>7.2599999999999998E-2</v>
       </c>
       <c r="L21">
         <v>0.25</v>
       </c>
       <c r="M21">
-        <v>0.0234</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>p8_agregado</t>
-        </is>
+        <v>2.3400000000000001E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
       <c r="B22">
-        <v>0.0201</v>
+        <v>2.01E-2</v>
       </c>
       <c r="C22">
-        <v>0.0106</v>
+        <v>1.06E-2</v>
       </c>
       <c r="D22">
-        <v>0.0346</v>
+        <v>3.4599999999999999E-2</v>
       </c>
       <c r="E22">
-        <v>0.2638</v>
+        <v>0.26379999999999998</v>
       </c>
       <c r="F22">
         <v>0.02</v>
       </c>
       <c r="G22">
-        <v>0.0499</v>
+        <v>4.99E-2</v>
       </c>
       <c r="H22">
-        <v>0.025</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="I22">
         <v>0.1517</v>
       </c>
       <c r="J22">
-        <v>0.043</v>
+        <v>4.2999999999999997E-2</v>
       </c>
       <c r="K22">
-        <v>0.0138</v>
+        <v>1.38E-2</v>
       </c>
       <c r="L22">
-        <v>0.019</v>
+        <v>1.9E-2</v>
       </c>
       <c r="M22">
-        <v>0.0436</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>p9_estrato3</t>
-        </is>
+        <v>4.36E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>34</v>
       </c>
       <c r="B23">
-        <v>0.0145</v>
+        <v>1.4500000000000001E-2</v>
       </c>
       <c r="C23">
-        <v>0.0139</v>
+        <v>1.3899999999999999E-2</v>
       </c>
       <c r="D23">
-        <v>0.0732</v>
+        <v>7.3200000000000001E-2</v>
       </c>
       <c r="E23">
-        <v>0.0291</v>
+        <v>2.9100000000000001E-2</v>
       </c>
       <c r="F23">
-        <v>0.0091</v>
+        <v>9.1000000000000004E-3</v>
       </c>
       <c r="G23">
-        <v>0.464</v>
+        <v>0.46400000000000002</v>
       </c>
       <c r="H23">
-        <v>0.0104</v>
+        <v>1.04E-2</v>
       </c>
       <c r="I23">
-        <v>0.0021</v>
+        <v>2.0999999999999999E-3</v>
       </c>
       <c r="J23">
-        <v>0.0176</v>
+        <v>1.7600000000000001E-2</v>
       </c>
       <c r="K23">
-        <v>0.0171</v>
+        <v>1.7100000000000001E-2</v>
       </c>
       <c r="L23">
         <v>0.2051</v>
       </c>
       <c r="M23">
-        <v>0.0101</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>p40</t>
-        </is>
+        <v>1.01E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>35</v>
       </c>
       <c r="B24">
-        <v>0.041</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="C24">
-        <v>0.1301</v>
+        <v>0.13009999999999999</v>
       </c>
       <c r="D24">
-        <v>0.0146</v>
+        <v>1.46E-2</v>
       </c>
       <c r="E24">
-        <v>0.07340000000000001</v>
+        <v>7.3400000000000007E-2</v>
       </c>
       <c r="F24">
-        <v>0.0236</v>
+        <v>2.3599999999999999E-2</v>
       </c>
       <c r="G24">
-        <v>0.1117</v>
+        <v>0.11169999999999999</v>
       </c>
       <c r="H24">
-        <v>0.2154</v>
+        <v>0.21540000000000001</v>
       </c>
       <c r="I24">
-        <v>0.0483</v>
+        <v>4.8300000000000003E-2</v>
       </c>
       <c r="J24">
-        <v>0.0448</v>
+        <v>4.48E-2</v>
       </c>
       <c r="K24">
-        <v>0.0115</v>
+        <v>1.15E-2</v>
       </c>
       <c r="L24">
-        <v>0.0455</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="M24">
-        <v>0.0598</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>p13</t>
-        </is>
-      </c>
-      <c r="B25">
-        <v>0.4045</v>
+        <v>5.9799999999999999E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A25" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="3">
+        <v>0.40450000000000003</v>
       </c>
       <c r="C25">
-        <v>0.0009</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="D25">
-        <v>0.5057</v>
+        <v>0.50570000000000004</v>
       </c>
       <c r="E25">
-        <v>0.1102</v>
+        <v>0.11020000000000001</v>
       </c>
       <c r="F25">
-        <v>0.009599999999999999</v>
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="G25">
-        <v>0.0089</v>
+        <v>8.8999999999999999E-3</v>
       </c>
       <c r="H25">
         <v>0.06</v>
       </c>
       <c r="I25">
-        <v>0.0654</v>
+        <v>6.54E-2</v>
       </c>
       <c r="J25">
-        <v>0.0292</v>
+        <v>2.92E-2</v>
       </c>
       <c r="K25">
         <v>0.1182</v>
       </c>
       <c r="L25">
-        <v>0.0212</v>
+        <v>2.12E-2</v>
       </c>
       <c r="M25">
         <v>0.1464</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>p14</t>
-        </is>
-      </c>
-      <c r="B26">
-        <v>0.522</v>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="2">
+        <v>0.52200000000000002</v>
       </c>
       <c r="C26">
-        <v>0.0027</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="D26">
-        <v>0.5667</v>
+        <v>0.56669999999999998</v>
       </c>
       <c r="E26">
-        <v>0.0107</v>
+        <v>1.0699999999999999E-2</v>
       </c>
       <c r="F26">
-        <v>0.0122</v>
+        <v>1.2200000000000001E-2</v>
       </c>
       <c r="G26">
-        <v>0.0059</v>
+        <v>5.8999999999999999E-3</v>
       </c>
       <c r="H26">
-        <v>0.028</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="I26">
-        <v>0.0761</v>
+        <v>7.6100000000000001E-2</v>
       </c>
       <c r="J26">
-        <v>0.0211</v>
+        <v>2.1100000000000001E-2</v>
       </c>
       <c r="K26">
         <v>0.1459</v>
       </c>
       <c r="L26">
-        <v>0.0292</v>
+        <v>2.92E-2</v>
       </c>
       <c r="M26">
-        <v>0.083</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>p15_autos_agregado</t>
-        </is>
+        <v>8.3000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>38</v>
       </c>
       <c r="B27">
-        <v>0.0251</v>
+        <v>2.5100000000000001E-2</v>
       </c>
       <c r="C27">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="D27">
         <v>0.4143</v>
       </c>
       <c r="E27">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="F27">
-        <v>0.0021</v>
+        <v>2.0999999999999999E-3</v>
       </c>
       <c r="G27">
-        <v>0.0563</v>
+        <v>5.6300000000000003E-2</v>
       </c>
       <c r="H27">
-        <v>0.0042</v>
+        <v>4.1999999999999997E-3</v>
       </c>
       <c r="I27">
-        <v>0.0129</v>
+        <v>1.29E-2</v>
       </c>
       <c r="J27">
-        <v>0.0387</v>
+        <v>3.8699999999999998E-2</v>
       </c>
       <c r="K27">
-        <v>0.3047</v>
+        <v>0.30470000000000003</v>
       </c>
       <c r="L27">
-        <v>0.0039</v>
+        <v>3.8999999999999998E-3</v>
       </c>
       <c r="M27">
-        <v>0.0013</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>p15_1_autos_propios_agregado</t>
-        </is>
+        <v>1.2999999999999999E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>39</v>
       </c>
       <c r="B28">
-        <v>0.0222</v>
+        <v>2.2200000000000001E-2</v>
       </c>
       <c r="C28">
-        <v>0.0012</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="D28">
         <v>0.5655</v>
       </c>
       <c r="E28">
-        <v>0.0008</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="F28">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="G28">
-        <v>0.0745</v>
+        <v>7.4499999999999997E-2</v>
       </c>
       <c r="H28">
-        <v>0.0009</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="I28">
-        <v>0.0026</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="J28">
-        <v>0.0008</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="K28">
-        <v>0.5306</v>
+        <v>0.53059999999999996</v>
       </c>
       <c r="L28">
-        <v>0.008200000000000001</v>
+        <v>8.2000000000000007E-3</v>
       </c>
       <c r="M28">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>p16_motos_agregado</t>
-        </is>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>40</v>
       </c>
       <c r="B29">
         <v>0.3962</v>
       </c>
       <c r="C29">
-        <v>0.0071</v>
+        <v>7.1000000000000004E-3</v>
       </c>
       <c r="D29">
-        <v>0.0033</v>
+        <v>3.3E-3</v>
       </c>
       <c r="E29">
-        <v>0.0227</v>
+        <v>2.2700000000000001E-2</v>
       </c>
       <c r="F29">
-        <v>0.0028</v>
+        <v>2.8E-3</v>
       </c>
       <c r="G29">
-        <v>0.0323</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="H29">
-        <v>0.0034</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="I29">
-        <v>0.0273</v>
+        <v>2.7300000000000001E-2</v>
       </c>
       <c r="J29">
-        <v>0.0025</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="K29">
-        <v>0.0038</v>
+        <v>3.8E-3</v>
       </c>
       <c r="L29">
-        <v>0.0721</v>
+        <v>7.2099999999999997E-2</v>
       </c>
       <c r="M29">
-        <v>0.0127</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>p16_1_motos_propias_agregado</t>
-        </is>
-      </c>
-      <c r="B30">
-        <v>0.6675</v>
+        <v>1.2699999999999999E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" s="2">
+        <v>0.66749999999999998</v>
       </c>
       <c r="C30">
-        <v>0.0034</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="D30">
         <v>0</v>
       </c>
       <c r="E30">
-        <v>0.0013</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="F30">
-        <v>0.0061</v>
+        <v>6.1000000000000004E-3</v>
       </c>
       <c r="G30">
-        <v>0.0041</v>
+        <v>4.1000000000000003E-3</v>
       </c>
       <c r="H30">
-        <v>0.0195</v>
+        <v>1.95E-2</v>
       </c>
       <c r="I30">
-        <v>0.0231</v>
+        <v>2.3099999999999999E-2</v>
       </c>
       <c r="J30">
-        <v>0.0039</v>
+        <v>3.8999999999999998E-3</v>
       </c>
       <c r="K30">
-        <v>0.0309</v>
+        <v>3.09E-2</v>
       </c>
       <c r="L30">
-        <v>0.0553</v>
+        <v>5.5300000000000002E-2</v>
       </c>
       <c r="M30">
-        <v>0.0054</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>p17_modo_agregado</t>
-        </is>
-      </c>
-      <c r="B31">
-        <v>0.8733</v>
+        <v>5.4000000000000003E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="2">
+        <v>0.87329999999999997</v>
       </c>
       <c r="C31">
-        <v>0.0165</v>
+        <v>1.6500000000000001E-2</v>
       </c>
       <c r="D31">
-        <v>0.7539</v>
+        <v>0.75390000000000001</v>
       </c>
       <c r="E31">
-        <v>0.0699</v>
+        <v>6.9900000000000004E-2</v>
       </c>
       <c r="F31">
-        <v>0.0074</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="G31">
-        <v>0.0308</v>
+        <v>3.0800000000000001E-2</v>
       </c>
       <c r="H31">
-        <v>0.0124</v>
+        <v>1.24E-2</v>
       </c>
       <c r="I31">
-        <v>0.0789</v>
+        <v>7.8899999999999998E-2</v>
       </c>
       <c r="J31">
-        <v>0.0435</v>
+        <v>4.3499999999999997E-2</v>
       </c>
       <c r="K31">
-        <v>0.0343</v>
+        <v>3.4299999999999997E-2</v>
       </c>
       <c r="L31">
-        <v>0.0083</v>
+        <v>8.3000000000000001E-3</v>
       </c>
       <c r="M31">
-        <v>0.08069999999999999</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>cilindraje_auto_agregado</t>
-        </is>
+        <v>8.0699999999999994E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>43</v>
       </c>
       <c r="B32">
-        <v>0.0065</v>
+        <v>6.4999999999999997E-3</v>
       </c>
       <c r="C32">
-        <v>0.0005</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="D32">
-        <v>0.7635</v>
+        <v>0.76349999999999996</v>
       </c>
       <c r="E32">
-        <v>0.0191</v>
+        <v>1.9099999999999999E-2</v>
       </c>
       <c r="F32">
-        <v>0.0175</v>
+        <v>1.7500000000000002E-2</v>
       </c>
       <c r="G32">
         <v>0.1263</v>
       </c>
       <c r="H32">
-        <v>0.0327</v>
+        <v>3.27E-2</v>
       </c>
       <c r="I32">
-        <v>0.0772</v>
+        <v>7.7200000000000005E-2</v>
       </c>
       <c r="J32">
-        <v>0.0196</v>
+        <v>1.9599999999999999E-2</v>
       </c>
       <c r="K32">
-        <v>0.5332</v>
+        <v>0.53320000000000001</v>
       </c>
       <c r="L32">
         <v>0.1163</v>
       </c>
       <c r="M32">
-        <v>0.0605</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>cilindraje_moto_agregado</t>
-        </is>
-      </c>
-      <c r="B33">
+        <v>6.0499999999999998E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B33" s="2">
         <v>0.874</v>
       </c>
       <c r="C33">
-        <v>0.0224</v>
+        <v>2.24E-2</v>
       </c>
       <c r="D33">
-        <v>0.0086</v>
+        <v>8.6E-3</v>
       </c>
       <c r="E33">
-        <v>0.0403</v>
+        <v>4.0300000000000002E-2</v>
       </c>
       <c r="F33">
-        <v>0.0145</v>
+        <v>1.4500000000000001E-2</v>
       </c>
       <c r="G33">
-        <v>0.1175</v>
+        <v>0.11749999999999999</v>
       </c>
       <c r="H33">
-        <v>0.0157</v>
+        <v>1.5699999999999999E-2</v>
       </c>
       <c r="I33">
-        <v>0.1233</v>
+        <v>0.12330000000000001</v>
       </c>
       <c r="J33">
         <v>0.1012</v>
       </c>
       <c r="K33">
-        <v>0.0204</v>
+        <v>2.0400000000000001E-2</v>
       </c>
       <c r="L33">
-        <v>0.0549</v>
+        <v>5.4899999999999997E-2</v>
       </c>
       <c r="M33">
-        <v>0.0398</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>modelo_vehiculo_agregado</t>
-        </is>
-      </c>
-      <c r="B34">
-        <v>0.7393999999999999</v>
+        <v>3.9800000000000002E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B34" s="2">
+        <v>0.73939999999999995</v>
       </c>
       <c r="C34">
-        <v>0.0293</v>
+        <v>2.93E-2</v>
       </c>
       <c r="D34">
-        <v>0.3413</v>
+        <v>0.34129999999999999</v>
       </c>
       <c r="E34">
-        <v>0.0285</v>
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="F34">
-        <v>0.0271</v>
+        <v>2.7099999999999999E-2</v>
       </c>
       <c r="G34">
-        <v>0.2169</v>
+        <v>0.21690000000000001</v>
       </c>
       <c r="H34">
-        <v>0.0464</v>
+        <v>4.6399999999999997E-2</v>
       </c>
       <c r="I34">
-        <v>0.1659</v>
+        <v>0.16589999999999999</v>
       </c>
       <c r="J34">
-        <v>0.09039999999999999</v>
+        <v>9.0399999999999994E-2</v>
       </c>
       <c r="K34">
         <v>0.1341</v>
       </c>
       <c r="L34">
-        <v>0.0743</v>
+        <v>7.4300000000000005E-2</v>
       </c>
       <c r="M34">
-        <v>0.08069999999999999</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>p19comuna</t>
-        </is>
+        <v>8.0699999999999994E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>46</v>
       </c>
       <c r="B35">
-        <v>0.0788</v>
+        <v>7.8799999999999995E-2</v>
       </c>
       <c r="C35">
-        <v>0.2597</v>
+        <v>0.25969999999999999</v>
       </c>
       <c r="D35">
-        <v>0.1194</v>
+        <v>0.11940000000000001</v>
       </c>
       <c r="E35">
         <v>0.1202</v>
       </c>
       <c r="F35">
-        <v>0.1674</v>
+        <v>0.16739999999999999</v>
       </c>
       <c r="G35">
-        <v>0.5505</v>
+        <v>0.55049999999999999</v>
       </c>
       <c r="H35">
-        <v>0.0502</v>
+        <v>5.0200000000000002E-2</v>
       </c>
       <c r="I35">
-        <v>0.08699999999999999</v>
+        <v>8.6999999999999994E-2</v>
       </c>
       <c r="J35">
-        <v>0.2716</v>
+        <v>0.27160000000000001</v>
       </c>
       <c r="K35">
         <v>0.1003</v>
       </c>
       <c r="L35">
-        <v>0.4018</v>
+        <v>0.40179999999999999</v>
       </c>
       <c r="M35">
         <v>0.371</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>p22</t>
-        </is>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>47</v>
       </c>
       <c r="B36">
-        <v>0.0356</v>
+        <v>3.56E-2</v>
       </c>
       <c r="C36">
-        <v>0.0461</v>
+        <v>4.6100000000000002E-2</v>
       </c>
       <c r="D36">
-        <v>0.0271</v>
+        <v>2.7099999999999999E-2</v>
       </c>
       <c r="E36">
-        <v>0.0529</v>
+        <v>5.2900000000000003E-2</v>
       </c>
       <c r="F36">
-        <v>0.0438</v>
+        <v>4.3799999999999999E-2</v>
       </c>
       <c r="G36">
-        <v>0.0572</v>
+        <v>5.7200000000000001E-2</v>
       </c>
       <c r="H36">
-        <v>0.0219</v>
+        <v>2.1899999999999999E-2</v>
       </c>
       <c r="I36">
-        <v>0.1869</v>
+        <v>0.18690000000000001</v>
       </c>
       <c r="J36">
-        <v>0.0309</v>
+        <v>3.09E-2</v>
       </c>
       <c r="K36">
-        <v>0.0524</v>
+        <v>5.2400000000000002E-2</v>
       </c>
       <c r="L36">
-        <v>0.0215</v>
+        <v>2.1499999999999998E-2</v>
       </c>
       <c r="M36">
-        <v>0.095</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>p23_agregado</t>
-        </is>
+        <v>9.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>48</v>
       </c>
       <c r="B37">
-        <v>0.1269</v>
+        <v>0.12690000000000001</v>
       </c>
       <c r="C37">
-        <v>0.009599999999999999</v>
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="D37">
-        <v>0.0499</v>
+        <v>4.99E-2</v>
       </c>
       <c r="E37">
-        <v>0.5309</v>
+        <v>0.53090000000000004</v>
       </c>
       <c r="F37">
-        <v>0.0569</v>
+        <v>5.6899999999999999E-2</v>
       </c>
       <c r="G37">
-        <v>0.0597</v>
+        <v>5.9700000000000003E-2</v>
       </c>
       <c r="H37">
-        <v>0.0301</v>
+        <v>3.0099999999999998E-2</v>
       </c>
       <c r="I37">
-        <v>0.4236</v>
+        <v>0.42359999999999998</v>
       </c>
       <c r="J37">
-        <v>0.06759999999999999</v>
+        <v>6.7599999999999993E-2</v>
       </c>
       <c r="K37">
-        <v>0.0416</v>
+        <v>4.1599999999999998E-2</v>
       </c>
       <c r="L37">
-        <v>0.0927</v>
+        <v>9.2700000000000005E-2</v>
       </c>
       <c r="M37">
         <v>0.1056</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>p26_agregado</t>
-        </is>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>49</v>
       </c>
       <c r="B38">
-        <v>0.1682</v>
+        <v>0.16819999999999999</v>
       </c>
       <c r="C38">
-        <v>0.0074</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="D38">
-        <v>0.0541</v>
+        <v>5.4100000000000002E-2</v>
       </c>
       <c r="E38">
-        <v>0.07920000000000001</v>
+        <v>7.9200000000000007E-2</v>
       </c>
       <c r="F38">
-        <v>0.0248</v>
+        <v>2.4799999999999999E-2</v>
       </c>
       <c r="G38">
         <v>0.1111</v>
       </c>
       <c r="H38">
-        <v>0.0765</v>
+        <v>7.6499999999999999E-2</v>
       </c>
       <c r="I38">
-        <v>0.0929</v>
+        <v>9.2899999999999996E-2</v>
       </c>
       <c r="J38">
-        <v>0.0594</v>
+        <v>5.9400000000000001E-2</v>
       </c>
       <c r="K38">
-        <v>0.015</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="L38">
         <v>0.1221</v>
@@ -2012,566 +2167,541 @@
         <v>0.2079</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>p29_modo_ideal_agregado</t>
-        </is>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>50</v>
       </c>
       <c r="B39">
-        <v>0.2609</v>
+        <v>0.26090000000000002</v>
       </c>
       <c r="C39">
-        <v>0.015</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="D39">
-        <v>0.08119999999999999</v>
+        <v>8.1199999999999994E-2</v>
       </c>
       <c r="E39">
-        <v>0.1795</v>
+        <v>0.17949999999999999</v>
       </c>
       <c r="F39">
-        <v>0.0145</v>
+        <v>1.4500000000000001E-2</v>
       </c>
       <c r="G39">
-        <v>0.0481</v>
+        <v>4.8099999999999997E-2</v>
       </c>
       <c r="H39">
-        <v>0.0294</v>
+        <v>2.9399999999999999E-2</v>
       </c>
       <c r="I39">
-        <v>0.058</v>
+        <v>5.8000000000000003E-2</v>
       </c>
       <c r="J39">
-        <v>0.1224</v>
+        <v>0.12239999999999999</v>
       </c>
       <c r="K39">
-        <v>0.053</v>
+        <v>5.2999999999999999E-2</v>
       </c>
       <c r="L39">
-        <v>0.09180000000000001</v>
+        <v>9.1800000000000007E-2</v>
       </c>
       <c r="M39">
-        <v>0.0531</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>p30_razon_no_uso_agregado</t>
-        </is>
+        <v>5.3100000000000001E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>51</v>
       </c>
       <c r="B40">
         <v>0.1116</v>
       </c>
       <c r="C40">
-        <v>0.017</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="D40">
-        <v>0.044</v>
+        <v>4.3999999999999997E-2</v>
       </c>
       <c r="E40">
-        <v>0.0199</v>
+        <v>1.9900000000000001E-2</v>
       </c>
       <c r="F40">
-        <v>0.0067</v>
+        <v>6.7000000000000002E-3</v>
       </c>
       <c r="G40">
-        <v>0.1259</v>
+        <v>0.12590000000000001</v>
       </c>
       <c r="H40">
-        <v>0.0659</v>
+        <v>6.59E-2</v>
       </c>
       <c r="I40">
-        <v>0.06569999999999999</v>
+        <v>6.5699999999999995E-2</v>
       </c>
       <c r="J40">
-        <v>0.083</v>
+        <v>8.3000000000000004E-2</v>
       </c>
       <c r="K40">
-        <v>0.0223</v>
+        <v>2.23E-2</v>
       </c>
       <c r="L40">
         <v>0.1108</v>
       </c>
       <c r="M40">
-        <v>0.1228</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>p31_fuente_contaminacion_agregada</t>
-        </is>
+        <v>0.12280000000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>52</v>
       </c>
       <c r="B41">
-        <v>0.0187</v>
+        <v>1.8700000000000001E-2</v>
       </c>
       <c r="C41">
-        <v>0.0382</v>
+        <v>3.8199999999999998E-2</v>
       </c>
       <c r="D41">
-        <v>0.011</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="E41">
-        <v>0.075</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="F41">
-        <v>0.0386</v>
+        <v>3.8600000000000002E-2</v>
       </c>
       <c r="G41">
         <v>0.1106</v>
       </c>
       <c r="H41">
-        <v>0.0206</v>
+        <v>2.06E-2</v>
       </c>
       <c r="I41">
-        <v>0.077</v>
+        <v>7.6999999999999999E-2</v>
       </c>
       <c r="J41">
-        <v>0.048</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="K41">
-        <v>0.0498</v>
+        <v>4.9799999999999997E-2</v>
       </c>
       <c r="L41">
-        <v>0.07679999999999999</v>
+        <v>7.6799999999999993E-2</v>
       </c>
       <c r="M41">
-        <v>0.0805</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>p33_modo_contaminante_agregado</t>
-        </is>
+        <v>8.0500000000000002E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>53</v>
       </c>
       <c r="B42">
-        <v>0.0318</v>
+        <v>3.1800000000000002E-2</v>
       </c>
       <c r="C42">
-        <v>0.0653</v>
+        <v>6.5299999999999997E-2</v>
       </c>
       <c r="D42">
-        <v>0.0059</v>
+        <v>5.8999999999999999E-3</v>
       </c>
       <c r="E42">
-        <v>0.0287</v>
+        <v>2.87E-2</v>
       </c>
       <c r="F42">
-        <v>0.0253</v>
+        <v>2.53E-2</v>
       </c>
       <c r="G42">
-        <v>0.1587</v>
+        <v>0.15870000000000001</v>
       </c>
       <c r="H42">
-        <v>0.0118</v>
+        <v>1.18E-2</v>
       </c>
       <c r="I42">
-        <v>0.0664</v>
+        <v>6.6400000000000001E-2</v>
       </c>
       <c r="J42">
-        <v>0.0153</v>
+        <v>1.5299999999999999E-2</v>
       </c>
       <c r="K42">
-        <v>0.0282</v>
+        <v>2.8199999999999999E-2</v>
       </c>
       <c r="L42">
         <v>0.1072</v>
       </c>
       <c r="M42">
-        <v>0.0572</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>p35_razon_agregada</t>
-        </is>
+        <v>5.7200000000000001E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>54</v>
       </c>
       <c r="B43">
-        <v>0.0195</v>
+        <v>1.95E-2</v>
       </c>
       <c r="C43">
-        <v>0.0157</v>
+        <v>1.5699999999999999E-2</v>
       </c>
       <c r="D43">
-        <v>0.0251</v>
+        <v>2.5100000000000001E-2</v>
       </c>
       <c r="E43">
-        <v>0.0335</v>
+        <v>3.3500000000000002E-2</v>
       </c>
       <c r="F43">
-        <v>0.0108</v>
+        <v>1.0800000000000001E-2</v>
       </c>
       <c r="G43">
         <v>0.1603</v>
       </c>
       <c r="H43">
-        <v>0.0466</v>
+        <v>4.6600000000000003E-2</v>
       </c>
       <c r="I43">
-        <v>0.048</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J43">
-        <v>0.0468</v>
+        <v>4.6800000000000001E-2</v>
       </c>
       <c r="K43">
-        <v>0.0163</v>
+        <v>1.6299999999999999E-2</v>
       </c>
       <c r="L43">
-        <v>0.0582</v>
+        <v>5.8200000000000002E-2</v>
       </c>
       <c r="M43">
-        <v>0.0648</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>p38p38_1</t>
-        </is>
+        <v>6.4799999999999996E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>55</v>
       </c>
       <c r="B44">
-        <v>0.0026</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="C44">
-        <v>0.8189</v>
+        <v>0.81889999999999996</v>
       </c>
       <c r="D44">
-        <v>0.0002</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="E44">
-        <v>0.0028</v>
+        <v>2.8E-3</v>
       </c>
       <c r="F44">
-        <v>0.0002</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="G44">
-        <v>0.0022</v>
+        <v>2.2000000000000001E-3</v>
       </c>
       <c r="H44">
-        <v>0.2855</v>
+        <v>0.28549999999999998</v>
       </c>
       <c r="I44">
-        <v>0.0025</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="J44">
-        <v>0.0062</v>
+        <v>6.1999999999999998E-3</v>
       </c>
       <c r="K44">
-        <v>0.0011</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="L44">
-        <v>0.0009</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="M44">
-        <v>0.0141</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>p38p38_2</t>
-        </is>
+        <v>1.41E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>56</v>
       </c>
       <c r="B45">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="C45">
-        <v>0.8989</v>
+        <v>0.89890000000000003</v>
       </c>
       <c r="D45">
-        <v>0.0011</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="E45">
-        <v>0.0132</v>
+        <v>1.32E-2</v>
       </c>
       <c r="F45">
         <v>0</v>
       </c>
       <c r="G45">
-        <v>0.0019</v>
+        <v>1.9E-3</v>
       </c>
       <c r="H45">
-        <v>0.6037</v>
+        <v>0.60370000000000001</v>
       </c>
       <c r="I45">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="J45">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="K45">
-        <v>0.0007</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="L45">
-        <v>0.0005</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="M45">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>p38p38_3</t>
-        </is>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>57</v>
       </c>
       <c r="B46">
-        <v>0.0025</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="C46">
-        <v>0.8324</v>
+        <v>0.83240000000000003</v>
       </c>
       <c r="D46">
-        <v>0.0021</v>
+        <v>2.0999999999999999E-3</v>
       </c>
       <c r="E46">
-        <v>0.0043</v>
+        <v>4.3E-3</v>
       </c>
       <c r="F46">
-        <v>0.0007</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="G46">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="H46">
-        <v>0.5838</v>
+        <v>0.58379999999999999</v>
       </c>
       <c r="I46">
-        <v>0.0016</v>
+        <v>1.6000000000000001E-3</v>
       </c>
       <c r="J46">
-        <v>0.0026</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="K46">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="L46">
-        <v>0.0053</v>
+        <v>5.3E-3</v>
       </c>
       <c r="M46">
-        <v>0.0115</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>p38p38_4</t>
-        </is>
+        <v>1.15E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>58</v>
       </c>
       <c r="B47">
-        <v>0.0362</v>
+        <v>3.6200000000000003E-2</v>
       </c>
       <c r="C47">
-        <v>0.6253</v>
+        <v>0.62529999999999997</v>
       </c>
       <c r="D47">
-        <v>0.0163</v>
+        <v>1.6299999999999999E-2</v>
       </c>
       <c r="E47">
-        <v>0.0168</v>
+        <v>1.6799999999999999E-2</v>
       </c>
       <c r="F47">
-        <v>0.017</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="G47">
-        <v>0.0074</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="H47">
-        <v>0.2579</v>
+        <v>0.25790000000000002</v>
       </c>
       <c r="I47">
         <v>0.05</v>
       </c>
       <c r="J47">
-        <v>0.0028</v>
+        <v>2.8E-3</v>
       </c>
       <c r="K47">
-        <v>0.0005</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="L47">
         <v>0</v>
       </c>
       <c r="M47">
-        <v>0.0356</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>p38p38_5</t>
-        </is>
+        <v>3.56E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>59</v>
       </c>
       <c r="B48">
-        <v>0.0028</v>
+        <v>2.8E-3</v>
       </c>
       <c r="C48">
-        <v>0.8956</v>
+        <v>0.89559999999999995</v>
       </c>
       <c r="D48">
-        <v>0.0012</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="E48">
-        <v>0.0005</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="F48">
-        <v>0.0008</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="G48">
-        <v>0.0126</v>
+        <v>1.26E-2</v>
       </c>
       <c r="H48">
-        <v>0.4813</v>
+        <v>0.48130000000000001</v>
       </c>
       <c r="I48">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="J48">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="K48">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="L48">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="M48">
-        <v>0.0012</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>p38p38_6</t>
-        </is>
+        <v>1.1999999999999999E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>60</v>
       </c>
       <c r="B49">
-        <v>0.0055</v>
+        <v>5.4999999999999997E-3</v>
       </c>
       <c r="C49">
-        <v>0.7884</v>
+        <v>0.78839999999999999</v>
       </c>
       <c r="D49">
-        <v>0.0019</v>
+        <v>1.9E-3</v>
       </c>
       <c r="E49">
-        <v>0.0369</v>
+        <v>3.6900000000000002E-2</v>
       </c>
       <c r="F49">
-        <v>0.0056</v>
+        <v>5.5999999999999999E-3</v>
       </c>
       <c r="G49">
-        <v>0.0015</v>
+        <v>1.5E-3</v>
       </c>
       <c r="H49">
-        <v>0.2388</v>
+        <v>0.23880000000000001</v>
       </c>
       <c r="I49">
-        <v>0.0139</v>
+        <v>1.3899999999999999E-2</v>
       </c>
       <c r="J49">
-        <v>0.0064</v>
+        <v>6.4000000000000003E-3</v>
       </c>
       <c r="K49">
-        <v>0.0028</v>
+        <v>2.8E-3</v>
       </c>
       <c r="L49">
-        <v>0.0013</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="M49">
-        <v>0.0008</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>p38p38_7</t>
-        </is>
+        <v>8.0000000000000004E-4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>61</v>
       </c>
       <c r="B50">
-        <v>0.0058</v>
+        <v>5.7999999999999996E-3</v>
       </c>
       <c r="C50">
-        <v>0.301</v>
+        <v>0.30099999999999999</v>
       </c>
       <c r="D50">
-        <v>0.0021</v>
+        <v>2.0999999999999999E-3</v>
       </c>
       <c r="E50">
-        <v>0.0031</v>
+        <v>3.0999999999999999E-3</v>
       </c>
       <c r="F50">
-        <v>0.0018</v>
+        <v>1.8E-3</v>
       </c>
       <c r="G50">
-        <v>0.0189</v>
+        <v>1.89E-2</v>
       </c>
       <c r="H50">
-        <v>0.0486</v>
+        <v>4.8599999999999997E-2</v>
       </c>
       <c r="I50">
-        <v>0.0774</v>
+        <v>7.7399999999999997E-2</v>
       </c>
       <c r="J50">
-        <v>0.0147</v>
+        <v>1.47E-2</v>
       </c>
       <c r="K50">
-        <v>0.0043</v>
+        <v>4.3E-3</v>
       </c>
       <c r="L50">
-        <v>0.0115</v>
+        <v>1.15E-2</v>
       </c>
       <c r="M50">
-        <v>0.0486</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>p38p38_99</t>
-        </is>
+        <v>4.8599999999999997E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>62</v>
       </c>
       <c r="B51">
-        <v>0.0258</v>
+        <v>2.58E-2</v>
       </c>
       <c r="C51">
-        <v>0.0251</v>
+        <v>2.5100000000000001E-2</v>
       </c>
       <c r="D51">
-        <v>0.0024</v>
+        <v>2.3999999999999998E-3</v>
       </c>
       <c r="E51">
-        <v>0.0097</v>
+        <v>9.7000000000000003E-3</v>
       </c>
       <c r="F51">
-        <v>0.0028</v>
+        <v>2.8E-3</v>
       </c>
       <c r="G51">
-        <v>0.0014</v>
+        <v>1.4E-3</v>
       </c>
       <c r="H51">
-        <v>0.0195</v>
+        <v>1.95E-2</v>
       </c>
       <c r="I51">
-        <v>0.0069</v>
+        <v>6.8999999999999999E-3</v>
       </c>
       <c r="J51">
-        <v>0.0182</v>
+        <v>1.8200000000000001E-2</v>
       </c>
       <c r="K51">
-        <v>0.0141</v>
+        <v>1.41E-2</v>
       </c>
       <c r="L51">
-        <v>0.0161</v>
+        <v>1.61E-2</v>
       </c>
       <c r="M51">
-        <v>0.1962</v>
+        <v>0.19620000000000001</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>